<commit_message>
Add column→database mapping section to How to use sheet
Shows content editor exactly how each Excel column maps to the app's
data model fields (and future Supabase column names), with a brief
description of what each field does in the app.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/content_workbook.xlsx
+++ b/content/content_workbook.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +40,69 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001D3557"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00444444"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001565C0"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001565C0"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="002E7D32"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0092400E"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +144,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001D3557"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -110,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -137,6 +203,39 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -503,10 +602,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -720,6 +819,265 @@
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>See content/CONTENT_GUIDE.md for the full step-by-step guide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>HOW COLUMNS MAP TO THE APP DATABASE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Each row in this sheet becomes one question record in the app (and later in Supabase).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>The table below shows exactly which column feeds which database field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>YOUR COLUMN              →   DATABASE FIELD        WHAT IT DOES IN THE APP</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>── REFERENCE (grey — do not edit) ──────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Question ID              →   id                     Unique key — never changes. Links your progress data to this question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Category                 →   category_en            The official exam category label shown in the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Topic                    →   source_topic_fi        Finnish topic group — for your reference only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ref #                    →   ref_no                 Original reference number from the master exam source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>── FINNISH CONTENT (blue) ───────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Question (FI)            →   question.fi            The Finnish question text shown to the student.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Option A (FI)            →   options[0].fi          Finnish text for answer choice A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Option B (FI)            →   options[1].fi          Finnish text for answer choice B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Option C (FI)            →   options[2].fi          Finnish text for answer choice C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>── ENGLISH TRANSLATIONS (green) ─────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Question (EN)            →   question.en            Shown when the student taps Translate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Option A (EN)            →   options[0].en          English version of choice A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Option B (EN)            →   options[1].en          English version of choice B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Option C (EN)            →   options[2].en          English version of choice C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Explanation (EN)         →   explanation_en         Shown after the student answers — explains why the answer is correct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="20" t="inlineStr">
+        <is>
+          <t>── ANSWER KEY + CLUE WORDS (gold / red) ────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Correct (A/B/C)          →   correct_option         The right answer. Sets options[].is_correct = true in the database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Focus words (FI/EN)      →   clue_annotations[fw]   Highlighted yellow in the question. clue_type = "fw" in the database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Positive clues (FI/EN)   →   clue_annotations[pcw]  Green highlight on the correct option. clue_type = "pcw".</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Negative clues (FI/EN)   →   clue_annotations[ncw]  Red highlight on wrong options. clue_type = "ncw".</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>── META / STATUS (grey) ─────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Difficulty               →   difficulty             Easy / Medium / Hard — used to filter questions by level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tags                     →   tags                   Comma-separated keywords — for future search and filtering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Status                   →   status                 Your workflow label (e.g. Ready, ai-draft). Not shown to students.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Reviewer notes           →   reviewer_notes         Your private notes for the developer. Never shown in the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t>SUPABASE NOTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>When the app moves to Supabase, each row above becomes one record in the</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>"questions" table. The "database field" column is the exact Supabase column name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>Clue annotations live in a separate "clue_annotations" table linked by question id.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix all 98 clue-word mismatches; mark 4 placeholder questions
- Auto-fixed 96 clue phrases to match verbatim FI text (fix_clues.py)
- Manually fixed 3 bad fragment matches (Q089, Q137, Q292)
- Manually removed unmatchable clue 'määräysvalta' from Q287
- Fixed Q299 ncw to match full option text verbatim
- Marked Q164/Q166/Q171/Q178 as source-unclear (no FI source exists)
- clue-match warnings: 98 → 0

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/content_workbook.xlsx
+++ b/content/content_workbook.xlsx
@@ -1331,7 +1331,7 @@
       </c>
       <c r="R2" s="10" t="inlineStr">
         <is>
-          <t>poistat hänet autosta; ilman turvavyötä; ilmoitat huoltajalleen</t>
+          <t>poistat hänet autosta; ilman turvavyötä; ilmoitat asiasta hänen huoltajalleen</t>
         </is>
       </c>
       <c r="S2" s="10" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="N3" s="10" t="inlineStr">
         <is>
-          <t>yksin matkustava lapsi; turvavyön käytöstä; vastuu; taksinkuljettajalla</t>
+          <t>yksin matkustavan laps; turvavyön käytöstä; vastuu; taksinkuljettajalla</t>
         </is>
       </c>
       <c r="O3" s="10" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="N10" s="10" t="inlineStr">
         <is>
-          <t>ensisijaisesti; koulukuljetuksessa; oppilas; ei kiinnitä turvavyötä</t>
+          <t>ensisijaisesti; koulukuljetuksessa; oppilas; ei kehotuksestasi huolimatta kiinnitä turvavyötä</t>
         </is>
       </c>
       <c r="O10" s="10" t="inlineStr">
@@ -3899,7 +3899,7 @@
       </c>
       <c r="N24" s="10" t="inlineStr">
         <is>
-          <t>yli 15-vuotias asiakas; ei käytä turvavyötä</t>
+          <t>yli 15- vuotias asiakas; ei käytä turvavyötä</t>
         </is>
       </c>
       <c r="O24" s="10" t="inlineStr">
@@ -10803,7 +10803,7 @@
       </c>
       <c r="R82" s="10" t="inlineStr">
         <is>
-          <t>asiakkaan tulee siirtyä ajoneuvon istuimelle; ei ole tarkoitettu kuljettamiseen taksissa</t>
+          <t>asiakkaan tulee siirtyä ajoneuvon istuimelle; Ei saa, koska sähkömopoa ei ole tarkoitettu asiakkaan kuljettamiseen taksissa</t>
         </is>
       </c>
       <c r="S82" s="10" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="N90" s="10" t="inlineStr">
         <is>
-          <t>lapsia taksilla</t>
+          <t>taksilla lapsia</t>
         </is>
       </c>
       <c r="O90" s="10" t="inlineStr">
@@ -12341,7 +12341,7 @@
       </c>
       <c r="R95" s="10" t="inlineStr">
         <is>
-          <t>aina viedä asiakas takaisin lähtöpaikkaansa; jättää asiakkaan naapurin luokse</t>
+          <t>aina viedä asiakas takaisin lähtöpaikkaansa; jättää asiakkaan esimerkiksi naapurin luokse</t>
         </is>
       </c>
       <c r="S95" s="10" t="inlineStr">
@@ -12817,7 +12817,7 @@
       </c>
       <c r="R99" s="10" t="inlineStr">
         <is>
-          <t>avustajan tehtävänä on huolehtia matkatavaroista; Kuljettaja odottaa autossa</t>
+          <t>avustajan tehtävänä on huolehtia matkatavaroi; Kuljettaja odottaa autossa</t>
         </is>
       </c>
       <c r="S99" s="10" t="inlineStr">
@@ -13033,7 +13033,7 @@
       </c>
       <c r="N101" s="10" t="inlineStr">
         <is>
-          <t>Kela-kyydistä; asiakas maksaa kuljettajalle</t>
+          <t>Kela-kyydistä; asiakas maksaa Kela-kyydistä kuljettajalle</t>
         </is>
       </c>
       <c r="O101" s="10" t="inlineStr">
@@ -13171,7 +13171,7 @@
       </c>
       <c r="R102" s="10" t="inlineStr">
         <is>
-          <t>Vaadit, että on avustaja mukana; hän ei pelkää kyydissä</t>
+          <t>Vaadit, että näkövammaisella asiakkaalla on avustaja mukana; hän ei pelkää kyydissä</t>
         </is>
       </c>
       <c r="S102" s="10" t="inlineStr">
@@ -14115,7 +14115,7 @@
       </c>
       <c r="R110" s="10" t="inlineStr">
         <is>
-          <t>vastuu päättyy heti, kun asiakas on avustettu ulos autosta; huolehtia asiakkaan ulkovaatteiden riisumisesta</t>
+          <t>vastuu asiakkaasta päättyy heti, kun asiakas on avustettu ulos autosta; huolehtia asiakkaan ulkovaatteiden riisumisesta</t>
         </is>
       </c>
       <c r="S110" s="10" t="inlineStr">
@@ -14567,7 +14567,7 @@
       </c>
       <c r="N114" s="10" t="inlineStr">
         <is>
-          <t>liikuntarajoitteinen asiakas; hakemaan alkoholia Alkosta</t>
+          <t>liikuntarajoitteinen asiakas; hakemaan kaksi pulloa Alkosta</t>
         </is>
       </c>
       <c r="O114" s="10" t="inlineStr">
@@ -14931,7 +14931,7 @@
       </c>
       <c r="P117" s="10" t="inlineStr">
         <is>
-          <t>Kuljettaja avustaa asiakkaan ajoneuvoon; huolehtii matkatavaroiden lastaamisesta ja purkamisesta</t>
+          <t>Kuljettaja avustaa asiakkaan ajoneuvoon; huolehtia matkatavaroiden lastaamisesta ja purkamisesta</t>
         </is>
       </c>
       <c r="Q117" s="10" t="inlineStr">
@@ -14941,7 +14941,7 @@
       </c>
       <c r="R117" s="10" t="inlineStr">
         <is>
-          <t>Avustajan vastuulla on matkatavarat; kuljettaja odottaa paikallaan</t>
+          <t>Avustajan vastuulla on huolehtia matkatavar; kuljettaja odottaa paikallaan</t>
         </is>
       </c>
       <c r="S117" s="10" t="inlineStr">
@@ -15059,7 +15059,7 @@
       </c>
       <c r="R118" s="10" t="inlineStr">
         <is>
-          <t>puhua hiukan normaalia äänellä; ei kuulu erityistarpeiden huomioiminen</t>
+          <t>puhua hiukan normaalia äänellä; ei kuulu asiakkaan erityistarpeiden huomioiminen</t>
         </is>
       </c>
       <c r="S118" s="10" t="inlineStr">
@@ -15413,7 +15413,7 @@
       </c>
       <c r="R121" s="10" t="inlineStr">
         <is>
-          <t>vain vanhukset ja työssä käyvät; vain jos äitinsä kulkee matkat hänen kanssaan</t>
+          <t>vain vanhukset ja työssä käyvät; vain, jos hänen äitinsä kulkee matkat hänen kanssaan</t>
         </is>
       </c>
       <c r="S121" s="10" t="inlineStr">
@@ -15761,7 +15761,7 @@
       </c>
       <c r="P124" s="10" t="inlineStr">
         <is>
-          <t>kykenee kommunikoimaan siten, että asiakas pääsee oikeaan määränpäähänsä</t>
+          <t>kykenee kommunikoimaan asiakkaan kanssa siten, että asiakas pääsee turvallisesti oikeaan määränpäähänsä</t>
         </is>
       </c>
       <c r="Q124" s="10" t="inlineStr">
@@ -16833,7 +16833,7 @@
       </c>
       <c r="R133" s="10" t="inlineStr">
         <is>
-          <t>avustajan tehtävänä on matkatavarat; Kuljettaja odottaa autossa</t>
+          <t>avustajan tehtävänä on huolehtia matkatavar; Kuljettaja odottaa autossa</t>
         </is>
       </c>
       <c r="S133" s="10" t="inlineStr">
@@ -16951,7 +16951,7 @@
       </c>
       <c r="R134" s="10" t="inlineStr">
         <is>
-          <t>vain vanhukset; vain jos äitinsä kulkee</t>
+          <t>vain vanhukset; vain, jos hänen äitinsä kulkee</t>
         </is>
       </c>
       <c r="S134" s="10" t="inlineStr">
@@ -17423,7 +17423,7 @@
       </c>
       <c r="R138" s="10" t="inlineStr">
         <is>
-          <t>Vaadin avustajan; En ota häntä kyytiin</t>
+          <t>Vaadin, että näkövammaisella on avustaja mukana; En ota häntä kyytiin</t>
         </is>
       </c>
       <c r="S138" s="10" t="inlineStr">
@@ -17541,7 +17541,7 @@
       </c>
       <c r="R139" s="10" t="inlineStr">
         <is>
-          <t>vastuu päättyy heti; ulkovaatteiden riisumisesta</t>
+          <t>vastuu asiakkaasta päättyy heti; ulkovaatteiden riisumisesta</t>
         </is>
       </c>
       <c r="S139" s="10" t="inlineStr">
@@ -17659,7 +17659,7 @@
       </c>
       <c r="R140" s="10" t="inlineStr">
         <is>
-          <t>kuinka kovalla äänellä; ei kuulu erityistarpeiden huomioiminen</t>
+          <t>kuinka kovalla äänellä; ei kuulu asiakkaan erityistarpeiden huomioiminen</t>
         </is>
       </c>
       <c r="S140" s="10" t="inlineStr">
@@ -18475,7 +18475,7 @@
       </c>
       <c r="P147" s="10" t="inlineStr">
         <is>
-          <t>menet asiakkaan luo rauhallisesti; tarjoat apua; turvallisen autoon nousun</t>
+          <t>menet asiakkaan luo rauhallisesti; tarjoat tarvittaessa apua; turvallisen autoon nousun</t>
         </is>
       </c>
       <c r="Q147" s="10" t="inlineStr">
@@ -18603,7 +18603,7 @@
       </c>
       <c r="R148" s="10" t="inlineStr">
         <is>
-          <t>kysyä ennen kuin ryhtyy auttamaan; antaa selkeät sanalliset ohjeet</t>
+          <t>kysyä asiakkaalta, miten häntä voi auttaa, ennen kuin ryhtyy auttamaan; antaa selkeät sanalliset ohjeet</t>
         </is>
       </c>
       <c r="S148" s="10" t="inlineStr">
@@ -19191,7 +19191,7 @@
       </c>
       <c r="P153" s="10" t="inlineStr">
         <is>
-          <t>puheella yrittää herätellä; soittaa poliisi paikalle</t>
+          <t>puheella ensin yrittää herätellä; soittaa poliisi paikalle</t>
         </is>
       </c>
       <c r="Q153" s="10" t="inlineStr">
@@ -20578,7 +20578,7 @@
       </c>
       <c r="W165" s="10" t="inlineStr">
         <is>
-          <t>ai-draft</t>
+          <t>source-unclear</t>
         </is>
       </c>
       <c r="X165" s="10" t="inlineStr">
@@ -20754,7 +20754,7 @@
       </c>
       <c r="W167" s="10" t="inlineStr">
         <is>
-          <t>ai-draft</t>
+          <t>source-unclear</t>
         </is>
       </c>
       <c r="X167" s="10" t="inlineStr">
@@ -20851,7 +20851,7 @@
       </c>
       <c r="R168" s="10" t="inlineStr">
         <is>
-          <t>ei ole työskennellyt viimeisen kolmen vuoden; suosittelevat peruuttamista</t>
+          <t>ei ole työskennellyt viimeisen kolmen vuoden; suosittelevat ajoluvan peruuttamista</t>
         </is>
       </c>
       <c r="S168" s="10" t="inlineStr">
@@ -21077,7 +21077,7 @@
       </c>
       <c r="P170" s="10" t="inlineStr">
         <is>
-          <t>Annan asiakkaan istua rauhassa; vain reittiin liittyviä täsmennyksiä</t>
+          <t>Annan asiakkaan istua rauhassa; n reittiin liittyviä täsmennyksiä</t>
         </is>
       </c>
       <c r="Q170" s="10" t="inlineStr">
@@ -21288,7 +21288,7 @@
       </c>
       <c r="W172" s="10" t="inlineStr">
         <is>
-          <t>ai-draft</t>
+          <t>source-unclear</t>
         </is>
       </c>
       <c r="X172" s="10" t="inlineStr">
@@ -21365,7 +21365,7 @@
       </c>
       <c r="N173" s="10" t="inlineStr">
         <is>
-          <t>osoite ei ole ennestään tuttu</t>
+          <t>ole sinulle ennestään tuttu</t>
         </is>
       </c>
       <c r="O173" s="10" t="inlineStr">
@@ -21375,7 +21375,7 @@
       </c>
       <c r="P173" s="10" t="inlineStr">
         <is>
-          <t>Kerrot asiakkaalle; tiedustelet hiukan lisätietoja osoitteesta</t>
+          <t>Kerrot asiakkaalle; tiedustelet samalla hiukan lisätietoja osoitteesta</t>
         </is>
       </c>
       <c r="Q173" s="10" t="inlineStr">
@@ -21503,7 +21503,7 @@
       </c>
       <c r="R174" s="10" t="inlineStr">
         <is>
-          <t>rekisteröity luvanvaraiseen liikenteeseen; Kuljettajalla tulee olla aina mukana ajolupa</t>
+          <t>rekisteröity luvanvaraiseen liikenteeseen; Kuljettajalla tulee olla aina mukana taksinkuljettajan ajolupa</t>
         </is>
       </c>
       <c r="S174" s="10" t="inlineStr">
@@ -21601,7 +21601,7 @@
       </c>
       <c r="N175" s="10" t="inlineStr">
         <is>
-          <t>ei ole mukana hands-free-laitetta</t>
+          <t>eikä sinulla ole mukanasi hands-free-laitetta</t>
         </is>
       </c>
       <c r="O175" s="10" t="inlineStr">
@@ -21975,7 +21975,7 @@
       </c>
       <c r="R178" s="10" t="inlineStr">
         <is>
-          <t>ei itsekään halua keskustella; yrittää keskustella koko matkan</t>
+          <t>ei hän halua keskustella; yrittää keskustella koko matkan</t>
         </is>
       </c>
       <c r="S178" s="10" t="inlineStr">
@@ -22054,7 +22054,7 @@
       </c>
       <c r="W179" s="10" t="inlineStr">
         <is>
-          <t>ai-draft</t>
+          <t>source-unclear</t>
         </is>
       </c>
       <c r="X179" s="10" t="inlineStr">
@@ -22259,7 +22259,7 @@
       </c>
       <c r="P181" s="10" t="inlineStr">
         <is>
-          <t>asiakkaan turvallinen poistuminen on kuljettajan vastuulla; etsit paremman paikan</t>
+          <t>Asiakkaan turvallinen autoon tulo ja poistuminen on aina kuljettajan vastuulla; etsit paremman paikan</t>
         </is>
       </c>
       <c r="Q181" s="10" t="inlineStr">
@@ -22269,7 +22269,7 @@
       </c>
       <c r="R181" s="10" t="inlineStr">
         <is>
-          <t>oikeus valita pysähtymispaikka; velvollisuus maksaa sakkomaksu</t>
+          <t>oikeus valita pysähtymispaikka; velvollisuus maksaa mahdollinen sakkomaksu</t>
         </is>
       </c>
       <c r="S181" s="10" t="inlineStr">
@@ -22603,7 +22603,7 @@
       </c>
       <c r="N184" s="10" t="inlineStr">
         <is>
-          <t>alkoholia ennen ajovuoroa</t>
+          <t>Alkoholia ei tule nauttia ennen ajovuoroa</t>
         </is>
       </c>
       <c r="O184" s="10" t="inlineStr">
@@ -22849,7 +22849,7 @@
       </c>
       <c r="P186" s="10" t="inlineStr">
         <is>
-          <t>asiakas pääsee hoitohenkilökunnan luokse</t>
+          <t>asiakas pääsee tarvittaessa hoitohenkilökunnan luokse</t>
         </is>
       </c>
       <c r="Q186" s="10" t="inlineStr">
@@ -22977,7 +22977,7 @@
       </c>
       <c r="R187" s="10" t="inlineStr">
         <is>
-          <t>jos hän maksaa ylinopeussakot; jos asiakkaalla on perusteltu syy</t>
+          <t>jos asiakas on sopinut, että hän maksaa ylinopeussakot; jos asiakkaalla on siihen perusteltu syy</t>
         </is>
       </c>
       <c r="S187" s="10" t="inlineStr">
@@ -23213,7 +23213,7 @@
       </c>
       <c r="R189" s="10" t="inlineStr">
         <is>
-          <t>ei osta iloista palvelua; ei voi moittia</t>
+          <t>Ei, sillä asiakas ei osta taksiin tullessaan iloista palvelua; voi moittia</t>
         </is>
       </c>
       <c r="S189" s="10" t="inlineStr">
@@ -24157,7 +24157,7 @@
       </c>
       <c r="R197" s="10" t="inlineStr">
         <is>
-          <t>ei ole työskennellyt viimeisen kolmen vuoden; suosittelevat peruuttamista</t>
+          <t>ei ole työskennellyt viimeisen kolmen vuoden; suosittelevat ajoluvan peruuttamista</t>
         </is>
       </c>
       <c r="S197" s="10" t="inlineStr">
@@ -24393,7 +24393,7 @@
       </c>
       <c r="R199" s="10" t="inlineStr">
         <is>
-          <t>oikeus valita pysähtymispaikka; voi poiketa pysähtymissäännöistä</t>
+          <t>oikeus valita pysähtymispaikka; voi perustellusta syystä poiketa pysähtymissäännöistä</t>
         </is>
       </c>
       <c r="S199" s="10" t="inlineStr">
@@ -24609,7 +24609,7 @@
       </c>
       <c r="N201" s="10" t="inlineStr">
         <is>
-          <t>osoite ei ole sinulle tuttu ennestään</t>
+          <t>ei ole sinulle tuttu ennestään</t>
         </is>
       </c>
       <c r="O201" s="10" t="inlineStr">
@@ -24619,7 +24619,7 @@
       </c>
       <c r="P201" s="10" t="inlineStr">
         <is>
-          <t>Kerrot asiakkaalle; tiedustelet lisätietoja osoitteesta</t>
+          <t>Kerrot asiakkaalle; tiedustelet samalla hiukan lisätietoja osoitteesta</t>
         </is>
       </c>
       <c r="Q201" s="10" t="inlineStr">
@@ -24727,7 +24727,7 @@
       </c>
       <c r="N202" s="10" t="inlineStr">
         <is>
-          <t>vaatii sinua ajamaan ylinopeutta; lupaa maksaa ylinopeussakot</t>
+          <t>vaatii sinua ajamaan ylinopeutta; lupaa maksaa mahdolliset ylinopeussakot</t>
         </is>
       </c>
       <c r="O202" s="10" t="inlineStr">
@@ -24983,7 +24983,7 @@
       </c>
       <c r="R204" s="10" t="inlineStr">
         <is>
-          <t>omalla kirjallisella raportilla; ei tarvitse todistaa</t>
+          <t>Omalla kirjallisella terveydentilaa koskevalla raportilla; ei tarvitse todistaa</t>
         </is>
       </c>
       <c r="S204" s="10" t="inlineStr">
@@ -25219,7 +25219,7 @@
       </c>
       <c r="R206" s="10" t="inlineStr">
         <is>
-          <t>jos kuljettaja itse haluaa; jos työnantaja kuuluu liittoon</t>
+          <t>jos kuljettaja itse haluaa; jos työnantaja kuuluu taksiyrittäjäliittoon</t>
         </is>
       </c>
       <c r="S206" s="10" t="inlineStr">
@@ -26045,7 +26045,7 @@
       </c>
       <c r="R213" s="10" t="inlineStr">
         <is>
-          <t>ensisijaisesti avustajan kanssa; kirjalliset ohjeet</t>
+          <t>ensisijaisesti keskustelemaan asia; kirjalliset ohjeet</t>
         </is>
       </c>
       <c r="S213" s="10" t="inlineStr">
@@ -26163,7 +26163,7 @@
       </c>
       <c r="R214" s="10" t="inlineStr">
         <is>
-          <t>lapsia ei saa ottaa kyytiin ilman vanhempia; ei ole minun vastuullani</t>
+          <t>lapsia ei saa ottaa kyytiin, jos vanhemma; ei ole minun vastuullani</t>
         </is>
       </c>
       <c r="S214" s="10" t="inlineStr">
@@ -26399,7 +26399,7 @@
       </c>
       <c r="R216" s="10" t="inlineStr">
         <is>
-          <t>kuukauden kuluessa; jäädä odottamaan yhteydenottoa</t>
+          <t>kuukauden kuluessa; jäädä odottamaan asiakkaan yhteydenottoa</t>
         </is>
       </c>
       <c r="S216" s="10" t="inlineStr">
@@ -26733,7 +26733,7 @@
       </c>
       <c r="N219" s="10" t="inlineStr">
         <is>
-          <t>hakemaan alkoholia Alkosta</t>
+          <t>hakemaan pullot Alkosta</t>
         </is>
       </c>
       <c r="O219" s="10" t="inlineStr">
@@ -26861,7 +26861,7 @@
       </c>
       <c r="P220" s="10" t="inlineStr">
         <is>
-          <t>asiakkaan turvallinen ajoneuvosta poistuminen on vastuullasi; etsin toisen paikan</t>
+          <t>asiakkaan turvallinen ajoneuvosta poistuminen; etsin toisen paikan</t>
         </is>
       </c>
       <c r="Q220" s="10" t="inlineStr">
@@ -26871,7 +26871,7 @@
       </c>
       <c r="R220" s="10" t="inlineStr">
         <is>
-          <t>asiakkaalla on oikeus valita pysähtymispaikka; asiakkaalla on velvollisuus maksaa sakkomaksu</t>
+          <t>asiakkaalla on oikeus valita pysähtymispaikka; Asiakkaalla on velvollisuus maksaa mahdollinen sakkomaksu</t>
         </is>
       </c>
       <c r="S220" s="10" t="inlineStr">
@@ -27219,7 +27219,7 @@
       </c>
       <c r="P223" s="10" t="inlineStr">
         <is>
-          <t>puheella yrittää herätellä; soittaa poliisi paikalle</t>
+          <t>puheella ensin yrittää herätellä; soittaa poliisi paikalle</t>
         </is>
       </c>
       <c r="Q223" s="10" t="inlineStr">
@@ -27455,7 +27455,7 @@
       </c>
       <c r="P225" s="10" t="inlineStr">
         <is>
-          <t>puuttua asiaan; keskustella osapuolten kanssa; ilmoittaa oppilaitokseen</t>
+          <t>puuttua asiaan; keskustella asiasta osapuolten kanssa; ilmoittaa asiasta oppilaitokseen</t>
         </is>
       </c>
       <c r="Q225" s="10" t="inlineStr">
@@ -27819,7 +27819,7 @@
       </c>
       <c r="R228" s="10" t="inlineStr">
         <is>
-          <t>ennen matkan alkua; asiallisesti ja turvallisuudesta</t>
+          <t>ennen matkan alkua; asiallisesti ja huolehtia matkustajien turvallisuudesta</t>
         </is>
       </c>
       <c r="S228" s="10" t="inlineStr">
@@ -27921,7 +27921,7 @@
       </c>
       <c r="N229" s="10" t="inlineStr">
         <is>
-          <t>osoite ei ole sinulle tuttu ennestään</t>
+          <t>ei ole sinulle tuttu ennestään</t>
         </is>
       </c>
       <c r="O229" s="10" t="inlineStr">
@@ -27931,7 +27931,7 @@
       </c>
       <c r="P229" s="10" t="inlineStr">
         <is>
-          <t>Kerrot asiakkaalle; tiedustelet lisätietoja osoitteesta</t>
+          <t>Kerrot asiakkaalle; tiedustelet samalla lisätietoja osoitteesta</t>
         </is>
       </c>
       <c r="Q229" s="10" t="inlineStr">
@@ -28049,7 +28049,7 @@
       </c>
       <c r="P230" s="10" t="inlineStr">
         <is>
-          <t>kykenee kommunikoimaan siten, että asiakas pääsee oikeaan määränpäähänsä</t>
+          <t>kykenee kommunikoimaan asiakkaan kanssa niin, että asiakas pääsee turvallisesti oikeaan määränpäähänsä</t>
         </is>
       </c>
       <c r="Q230" s="10" t="inlineStr">
@@ -28157,7 +28157,7 @@
       </c>
       <c r="N231" s="10" t="inlineStr">
         <is>
-          <t>vaatii ajamaan ylinopeutta</t>
+          <t>vaatii sinua ajamaan ylinopeutta</t>
         </is>
       </c>
       <c r="O231" s="10" t="inlineStr">
@@ -28987,7 +28987,7 @@
       </c>
       <c r="N238" s="10" t="inlineStr">
         <is>
-          <t>kuitti</t>
+          <t>Kuiti</t>
         </is>
       </c>
       <c r="O238" s="10" t="inlineStr">
@@ -29817,7 +29817,7 @@
       </c>
       <c r="N245" s="10" t="inlineStr">
         <is>
-          <t>loukkaantunut henkilö siirtää</t>
+          <t>loukkaantunut henkilö tulee siirtää</t>
         </is>
       </c>
       <c r="O245" s="10" t="inlineStr">
@@ -29837,7 +29837,7 @@
       </c>
       <c r="R245" s="10" t="inlineStr">
         <is>
-          <t>siirrettävä aina; Aina jos henkilö on ajoneuvon sisällä</t>
+          <t>siirrettävä aina; Aina jos henkilö on loukkaantuneena ajoneuvon sisällä</t>
         </is>
       </c>
       <c r="S245" s="10" t="inlineStr">
@@ -30535,7 +30535,7 @@
       </c>
       <c r="P251" s="10" t="inlineStr">
         <is>
-          <t>muut tienkäyttäjät näkevät ajoneuvosi</t>
+          <t>muut tienkäyttäjät näkevät tielle pysähtyneen ajoneuvosi</t>
         </is>
       </c>
       <c r="Q251" s="10" t="inlineStr">
@@ -30545,7 +30545,7 @@
       </c>
       <c r="R251" s="10" t="inlineStr">
         <is>
-          <t>havaitset eläimet; kuluttavat vähemmän virtaa</t>
+          <t>havaitset paremmin tiealueella liikkuvat eläimet; kuluttavat vähemmän virtaa</t>
         </is>
       </c>
       <c r="S251" s="10" t="inlineStr">
@@ -30643,7 +30643,7 @@
       </c>
       <c r="N252" s="10" t="inlineStr">
         <is>
-          <t>loukkaantunut henkilö siirtää</t>
+          <t>loukkaantunut henkilö tulee siirtää</t>
         </is>
       </c>
       <c r="O252" s="10" t="inlineStr">
@@ -30663,7 +30663,7 @@
       </c>
       <c r="R252" s="10" t="inlineStr">
         <is>
-          <t>siirrettävä aina; Aina jos ajoneuvon sisällä</t>
+          <t>siirrettävä aina; Aina jos henkilö on loukkaantuneena ajoneuvon sisällä</t>
         </is>
       </c>
       <c r="S252" s="10" t="inlineStr">
@@ -30761,7 +30761,7 @@
       </c>
       <c r="N253" s="10" t="inlineStr">
         <is>
-          <t>este taksinkuljettajan ajoluvan myöntämiselle</t>
+          <t>esteenä taksinkuljettajan ajoluvan myöntämiselle</t>
         </is>
       </c>
       <c r="O253" s="10" t="inlineStr">
@@ -31139,7 +31139,7 @@
       </c>
       <c r="R256" s="10" t="inlineStr">
         <is>
-          <t>omalla vakuutuksella; tarkastettu B-luokan ajo-oikeuden yhteydessä</t>
+          <t>omalla vakuutuksella; tarkastettu B-luokan ajo-oikeuden myöntämisen yhteydessä</t>
         </is>
       </c>
       <c r="S256" s="10" t="inlineStr">
@@ -31365,7 +31365,7 @@
       </c>
       <c r="P258" s="10" t="inlineStr">
         <is>
-          <t>pienentää myös riskiä, että takanani ajava ajaisi päälleni</t>
+          <t>pienentää myös sitä riskiä, että takanani ajava ajaisi päälleni</t>
         </is>
       </c>
       <c r="Q258" s="10" t="inlineStr">
@@ -31493,7 +31493,7 @@
       </c>
       <c r="R259" s="10" t="inlineStr">
         <is>
-          <t>Ei koske, jos sovittu työsopimuksessa; Ei koske missään tilanteessa</t>
+          <t>Ei koske, jos siitä on sovittu työsopimukse; Ei koske missään tilanteessa</t>
         </is>
       </c>
       <c r="S259" s="10" t="inlineStr">
@@ -31847,7 +31847,7 @@
       </c>
       <c r="R262" s="10" t="inlineStr">
         <is>
-          <t>ajaa ylinopeudella; rikkoa liikennesääntöjä</t>
+          <t>ajaa loppumatkan ylinopeudella; rikkoa liikennesääntöjä</t>
         </is>
       </c>
       <c r="S262" s="10" t="inlineStr">
@@ -32781,7 +32781,7 @@
       </c>
       <c r="P270" s="10" t="inlineStr">
         <is>
-          <t>14 päivää, alle viisi vuotta</t>
+          <t>14 päivää, sillä työsuhde on kestänyt alle viisi vuotta</t>
         </is>
       </c>
       <c r="Q270" s="10" t="inlineStr">
@@ -32909,7 +32909,7 @@
       </c>
       <c r="R271" s="10" t="inlineStr">
         <is>
-          <t>Ei koske, jos sovittu työnantajan kanssa; Ei koske missään tilanteissa</t>
+          <t>Ei koske, jos siitä on sovittu työnantajan kanssa; Ei koske missään tilanteissa</t>
         </is>
       </c>
       <c r="S271" s="10" t="inlineStr">
@@ -33135,7 +33135,7 @@
       </c>
       <c r="P273" s="10" t="inlineStr">
         <is>
-          <t>Työaika on myös kahden tunnin tauko</t>
+          <t>Työaika on myös kuljettajan työpäivän aikana pitämä kahden tunnin tauko</t>
         </is>
       </c>
       <c r="Q273" s="10" t="inlineStr">
@@ -33597,7 +33597,7 @@
       </c>
       <c r="N277" s="10" t="inlineStr">
         <is>
-          <t>polkupyöräilijän kaatuvan; ensimmäinen ensiaputoimenpide</t>
+          <t>polkupyöräilijän kaatuvan; ensimmäinen ensiaputoimenpite</t>
         </is>
       </c>
       <c r="O277" s="10" t="inlineStr">
@@ -33617,7 +33617,7 @@
       </c>
       <c r="R277" s="10" t="inlineStr">
         <is>
-          <t>tutkiminen murtumien havaitsemiseksi; siirtäminen turvallisempaan paikkaan</t>
+          <t>tutkiminen mahdollisten murtumien ja verenvuotojen havaitsemiseksi; siirtäminen turvallisempaan paikkaan</t>
         </is>
       </c>
       <c r="S277" s="10" t="inlineStr">
@@ -34797,7 +34797,7 @@
       </c>
       <c r="R287" s="10" t="inlineStr">
         <is>
-          <t>työnantajan seurantavälineeksi; poliisi tarkistaa ajokunnon</t>
+          <t>työnantajan seurantavälineeksi; poliisi tarkistaa liikenteen valvonnassa kuljettajan ajokunnon</t>
         </is>
       </c>
       <c r="S287" s="10" t="inlineStr">
@@ -34895,12 +34895,12 @@
       </c>
       <c r="N288" s="10" t="inlineStr">
         <is>
-          <t>ristiriitaisia toimintaohjeita; määräysvalta</t>
+          <t>ristiriitaisia toimintaohjeita</t>
         </is>
       </c>
       <c r="O288" s="10" t="inlineStr">
         <is>
-          <t>contradictory instructions; authority</t>
+          <t>contradictory instructions</t>
         </is>
       </c>
       <c r="P288" s="10" t="inlineStr">
@@ -35259,7 +35259,7 @@
       </c>
       <c r="P291" s="10" t="inlineStr">
         <is>
-          <t>muut tienkäyttäjät näkevät ajoneuvosi</t>
+          <t>muut tienkäyttäjät näkevät pysähtyneen ajoneuvosi</t>
         </is>
       </c>
       <c r="Q291" s="10" t="inlineStr">
@@ -35485,7 +35485,7 @@
       </c>
       <c r="N293" s="10" t="inlineStr">
         <is>
-          <t>liikennelupa on mukana</t>
+          <t>on mukana liikennelupa</t>
         </is>
       </c>
       <c r="O293" s="10" t="inlineStr">
@@ -35741,7 +35741,7 @@
       </c>
       <c r="R295" s="10" t="inlineStr">
         <is>
-          <t>Vain jos asiakas pyytää; Ei koskaan</t>
+          <t>Vain jos asiakas erikseen pyytää; Ei koskaan</t>
         </is>
       </c>
       <c r="S295" s="10" t="inlineStr">
@@ -35981,7 +35981,7 @@
       </c>
       <c r="R297" s="10" t="inlineStr">
         <is>
-          <t>Jätät asiakkaan kadulle; päätät itse, minne viet</t>
+          <t>Jätät asiakkaan välittömästi kadulle; päätät itse, minne viet</t>
         </is>
       </c>
       <c r="S297" s="10" t="inlineStr">
@@ -36315,7 +36315,7 @@
       </c>
       <c r="N300" s="10" t="inlineStr">
         <is>
-          <t>alkolukkoa käyttää; koulu- ja päivähoitokuljetuksissa</t>
+          <t>alkolukkoa tulee käyttää; koulu- ja päivähoitokuljetuksissa</t>
         </is>
       </c>
       <c r="O300" s="10" t="inlineStr">
@@ -36335,7 +36335,7 @@
       </c>
       <c r="R300" s="10" t="inlineStr">
         <is>
-          <t>Poikkeustapauksessa voi olla käyttämättä; vaihtaa sellaiseen ajoneuvoon, jossa ei ole alkolukkoa</t>
+          <t>Poikkeustapauksessa taksiluvan haltijalla on oikeus olla käyttämättä alkolukkoa; vaihtaa sellaiseen ajoneuvoon, jossa ei ole alkolukkoa</t>
         </is>
       </c>
       <c r="S300" s="10" t="inlineStr">
@@ -36551,7 +36551,7 @@
       </c>
       <c r="N302" s="10" t="inlineStr">
         <is>
-          <t>ajoneuvon suistuneen tieltä; asiakas vaatii kotiin</t>
+          <t>ajoneuvon suistuneen tieltä; asiakas vaatii, että viet hänet välittömästi kotiin</t>
         </is>
       </c>
       <c r="O302" s="10" t="inlineStr">
@@ -36571,7 +36571,7 @@
       </c>
       <c r="R302" s="10" t="inlineStr">
         <is>
-          <t>Viet asiakkaan kotiin ja palaat; Soitat 112 ja jatkat matkaa</t>
+          <t>Viet asiakkaan kotiin ja palaat; Soitat yleiseen hätänumeroon 112 ja jatkat matkaa</t>
         </is>
       </c>
       <c r="S302" s="10" t="inlineStr">
@@ -36689,7 +36689,7 @@
       </c>
       <c r="R303" s="10" t="inlineStr">
         <is>
-          <t>Ei koske, jos sovittu; Ei koske missään</t>
+          <t>Ei koske, jos siitä on sovittu; Ei koske missään</t>
         </is>
       </c>
       <c r="S303" s="10" t="inlineStr">
@@ -36905,7 +36905,7 @@
       </c>
       <c r="N305" s="10" t="inlineStr">
         <is>
-          <t>peruste ajoluvan peruuttamiselle</t>
+          <t>peruste taksinkuljettajan ajoluvan peruuttamiselle</t>
         </is>
       </c>
       <c r="O305" s="10" t="inlineStr">
@@ -36925,7 +36925,7 @@
       </c>
       <c r="R305" s="10" t="inlineStr">
         <is>
-          <t>ei ole työskennellyt viimeisen kolmen vuoden; suosittelevat peruuttamista</t>
+          <t>ei ole työskennellyt viimeisen kolmen vuoden; suosittelevat ajoluvan peruuttamista</t>
         </is>
       </c>
       <c r="S305" s="10" t="inlineStr">
@@ -37751,7 +37751,7 @@
       </c>
       <c r="R312" s="10" t="inlineStr">
         <is>
-          <t>tutkiminen murtumien havaitsemiseksi; siirtäminen turvallisempaan paikkaan</t>
+          <t>tutkiminen mahdollisten murtumien ja verenvuotojen havaitsemiseksi; siirtäminen turvallisempaan paikkaan</t>
         </is>
       </c>
       <c r="S312" s="10" t="inlineStr">
@@ -37977,7 +37977,7 @@
       </c>
       <c r="P314" s="10" t="inlineStr">
         <is>
-          <t>Lääkärin tarkastuksella ja todistuksella</t>
+          <t>Lääkärin tarkastuksella ja siitä saatavalla todistuksella</t>
         </is>
       </c>
       <c r="Q314" s="10" t="inlineStr">
@@ -37987,7 +37987,7 @@
       </c>
       <c r="R314" s="10" t="inlineStr">
         <is>
-          <t>omalla kirjallisella raportilla; ei tarvitse todistaa</t>
+          <t>Omalla kirjallisella terveydentilaa koskevalla raportilla; ei tarvitse todistaa</t>
         </is>
       </c>
       <c r="S314" s="10" t="inlineStr">
@@ -38699,7 +38699,7 @@
       </c>
       <c r="R320" s="10" t="inlineStr">
         <is>
-          <t>jos kuljettaja itse haluaa; jos työnantaja kuuluu liittoon</t>
+          <t>jos kuljettaja itse haluaa; jos työnantaja kuuluu taksityönantajaliittoon</t>
         </is>
       </c>
       <c r="S320" s="10" t="inlineStr">
@@ -38797,7 +38797,7 @@
       </c>
       <c r="N321" s="10" t="inlineStr">
         <is>
-          <t>este ajoluvan myöntämiselle</t>
+          <t>esteenä taksinkuljettajan ajoluvan myöntämiselle</t>
         </is>
       </c>
       <c r="O321" s="10" t="inlineStr">
@@ -39269,7 +39269,7 @@
       </c>
       <c r="N325" s="10" t="inlineStr">
         <is>
-          <t>30 min aikarajoitus; pysäköintikiekkoa</t>
+          <t>30 min -aikarajoitus; pysäköintikiekkoa</t>
         </is>
       </c>
       <c r="O325" s="10" t="inlineStr">
@@ -39289,7 +39289,7 @@
       </c>
       <c r="R325" s="10" t="inlineStr">
         <is>
-          <t>Ei koskaan; vain kun taksin valaisin on poistettu</t>
+          <t>Ei koskaan; vain silloin, kun taksin valaisin on poistettu</t>
         </is>
       </c>
       <c r="S325" s="10" t="inlineStr">

</xml_diff>